<commit_message>
edited economy.xlsx to have correct ranges for time_index2009 and 2014 and _projection, and for all data to stop at 2014. changed _ext_lookup_historic_final_energy_intensity in pymedeas for world sim to go all the way to 2014 instead of 2009. this will likely make the 14sectors_cat default sim to crash. not sure if these fixes help because same error when running 16sectors_qc pymedeas_w sim.
</commit_message>
<xml_diff>
--- a/models/16sectors_qc/climate.xlsx
+++ b/models/16sectors_qc/climate.xlsx
@@ -157,6 +157,23 @@
     <definedName name="year_ccs_tech" localSheetId="1">World!$C$151:$N$151</definedName>
     <definedName name="year_emissions" localSheetId="1">World!$D$94:$P$94</definedName>
     <definedName name="years_process_emissions" localSheetId="1">World!$C$208:$AD$208</definedName>
+    <definedName name="ccs_tech_share_Households" localSheetId="1">World!$C$152:$N$154</definedName>
+    <definedName name="ccs_tech_share_Agriculture_Forestry" localSheetId="1">World!$C$155:$N$157</definedName>
+    <definedName name="ccs_tech_share_Manufacturing" localSheetId="1">World!$C$158:$N$160</definedName>
+    <definedName name="ccs_tech_share_Mining" localSheetId="1">World!$C$161:$N$163</definedName>
+    <definedName name="ccs_tech_share_Utilities" localSheetId="1">World!$C$164:$N$166</definedName>
+    <definedName name="ccs_tech_share_Construction" localSheetId="1">World!$C$167:$N$169</definedName>
+    <definedName name="ccs_tech_share_Motor_Vehicles" localSheetId="1">World!$C$170:$N$172</definedName>
+    <definedName name="ccs_tech_share_Wholesale_Trade" localSheetId="1">World!$C$173:$N$175</definedName>
+    <definedName name="ccs_tech_share_Retail_Trade" localSheetId="1">World!$C$176:$N$178</definedName>
+    <definedName name="ccs_tech_share_Hotels_and_Restaurants" localSheetId="1">World!$C$179:$N$181</definedName>
+    <definedName name="ccs_tech_share_Transport" localSheetId="1">World!$C$182:$N$184</definedName>
+    <definedName name="ccs_tech_share_Post_and_Telecomm" localSheetId="1">World!$C$185:$N$187</definedName>
+    <definedName name="ccs_tech_share_Offices" localSheetId="1">World!$C$188:$N$190</definedName>
+    <definedName name="ccs_tech_share_Education" localSheetId="1">World!$C$191:$N$193</definedName>
+    <definedName name="ccs_tech_share_Health_and_Social_work" localSheetId="1">World!$C$194:$N$196</definedName>
+    <definedName name="ccs_tech_share_Other_Community_Social_and_Personal_Services" localSheetId="1">World!$C$197:$N$199</definedName>
+    <definedName name="ccs_tech_share_Private_Households" localSheetId="1">World!$C$200:$N$202</definedName>
     <definedName name="ccs_tech_share" localSheetId="2">Europe!$C$59:$N$103</definedName>
     <definedName name="ccs_tech_share_agr" localSheetId="2">Europe!$C$62:$N$64</definedName>
     <definedName name="ccs_tech_share_coke" localSheetId="2">Europe!$C$74:$N$76</definedName>
@@ -192,6 +209,23 @@
     <definedName name="year_ccs_tech" localSheetId="2">Europe!$C$58:$N$58</definedName>
     <definedName name="year_emissions" localSheetId="2">Europe!$D$1:$P$1</definedName>
     <definedName name="years_process_emissions" localSheetId="2">Europe!$C$115:$AD$115</definedName>
+    <definedName name="ccs_tech_share_Households" localSheetId="2">Europe!$C$59:$N$61</definedName>
+    <definedName name="ccs_tech_share_Agriculture_Forestry" localSheetId="2">Europe!$C$62:$N$64</definedName>
+    <definedName name="ccs_tech_share_Manufacturing" localSheetId="2">Europe!$C$65:$N$67</definedName>
+    <definedName name="ccs_tech_share_Mining" localSheetId="2">Europe!$C$68:$N$70</definedName>
+    <definedName name="ccs_tech_share_Utilities" localSheetId="2">Europe!$C$71:$N$73</definedName>
+    <definedName name="ccs_tech_share_Construction" localSheetId="2">Europe!$C$74:$N$76</definedName>
+    <definedName name="ccs_tech_share_Motor_Vehicles" localSheetId="2">Europe!$C$77:$N$79</definedName>
+    <definedName name="ccs_tech_share_Wholesale_Trade" localSheetId="2">Europe!$C$80:$N$82</definedName>
+    <definedName name="ccs_tech_share_Retail_Trade" localSheetId="2">Europe!$C$83:$N$85</definedName>
+    <definedName name="ccs_tech_share_Hotels_and_Restaurants" localSheetId="2">Europe!$C$86:$N$88</definedName>
+    <definedName name="ccs_tech_share_Transport" localSheetId="2">Europe!$C$89:$N$91</definedName>
+    <definedName name="ccs_tech_share_Post_and_Telecomm" localSheetId="2">Europe!$C$92:$N$94</definedName>
+    <definedName name="ccs_tech_share_Offices" localSheetId="2">Europe!$C$95:$N$97</definedName>
+    <definedName name="ccs_tech_share_Education" localSheetId="2">Europe!$C$98:$N$100</definedName>
+    <definedName name="ccs_tech_share_Health_and_Social_work" localSheetId="2">Europe!$C$101:$N$103</definedName>
+    <definedName name="ccs_tech_share_Other_Community_Social_and_Personal_Services" localSheetId="2">Europe!$C$104:$N$106</definedName>
+    <definedName name="ccs_tech_share_Private_Households" localSheetId="2">Europe!$C$107:$N$109</definedName>
     <definedName name="ccs_tech_share_agr" localSheetId="3">Catalonia!$C$68:$N$70</definedName>
     <definedName name="ccs_tech_share_coke" localSheetId="3">Catalonia!$C$80:$N$82</definedName>
     <definedName name="ccs_tech_share_cons" localSheetId="3">Catalonia!$C$89:$N$91</definedName>
@@ -230,40 +264,6 @@
     <definedName name="year_ccs_tech" localSheetId="3">Catalonia!$C$64:$N$64</definedName>
     <definedName name="year_emissions" localSheetId="3">Catalonia!$D$1:$P$1</definedName>
     <definedName name="years_process_emissions" localSheetId="3">Catalonia!$C$117:$AC$117</definedName>
-    <definedName name="ccs_tech_share_Households" localSheetId="1">World!$C$152:$N$154</definedName>
-    <definedName name="ccs_tech_share_Agriculture_Forestry" localSheetId="1">World!$C$155:$N$157</definedName>
-    <definedName name="ccs_tech_share_Manufacturing" localSheetId="1">World!$C$158:$N$160</definedName>
-    <definedName name="ccs_tech_share_Mining" localSheetId="1">World!$C$161:$N$163</definedName>
-    <definedName name="ccs_tech_share_Utilities" localSheetId="1">World!$C$164:$N$166</definedName>
-    <definedName name="ccs_tech_share_Construction" localSheetId="1">World!$C$167:$N$169</definedName>
-    <definedName name="ccs_tech_share_Motor_Vehicles" localSheetId="1">World!$C$170:$N$172</definedName>
-    <definedName name="ccs_tech_share_Wholesale_Trade" localSheetId="1">World!$C$173:$N$175</definedName>
-    <definedName name="ccs_tech_share_Retail_Trade" localSheetId="1">World!$C$176:$N$178</definedName>
-    <definedName name="ccs_tech_share_Hotels_and_Restaurants" localSheetId="1">World!$C$179:$N$181</definedName>
-    <definedName name="ccs_tech_share_Transport" localSheetId="1">World!$C$182:$N$184</definedName>
-    <definedName name="ccs_tech_share_Post_and_Telecomm" localSheetId="1">World!$C$185:$N$187</definedName>
-    <definedName name="ccs_tech_share_Offices" localSheetId="1">World!$C$188:$N$190</definedName>
-    <definedName name="ccs_tech_share_Education" localSheetId="1">World!$C$191:$N$193</definedName>
-    <definedName name="ccs_tech_share_Health_and_Social_work" localSheetId="1">World!$C$194:$N$196</definedName>
-    <definedName name="ccs_tech_share_Other_Community_Social_and_Personal_Services" localSheetId="1">World!$C$197:$N$199</definedName>
-    <definedName name="ccs_tech_share_Private_Households" localSheetId="1">World!$C$200:$N$202</definedName>
-    <definedName name="ccs_tech_share_Households" localSheetId="2">Europe!$C$59:$N$61</definedName>
-    <definedName name="ccs_tech_share_Agriculture_Forestry" localSheetId="2">Europe!$C$62:$N$64</definedName>
-    <definedName name="ccs_tech_share_Manufacturing" localSheetId="2">Europe!$C$65:$N$67</definedName>
-    <definedName name="ccs_tech_share_Mining" localSheetId="2">Europe!$C$68:$N$70</definedName>
-    <definedName name="ccs_tech_share_Utilities" localSheetId="2">Europe!$C$71:$N$73</definedName>
-    <definedName name="ccs_tech_share_Construction" localSheetId="2">Europe!$C$74:$N$76</definedName>
-    <definedName name="ccs_tech_share_Motor_Vehicles" localSheetId="2">Europe!$C$77:$N$79</definedName>
-    <definedName name="ccs_tech_share_Wholesale_Trade" localSheetId="2">Europe!$C$80:$N$82</definedName>
-    <definedName name="ccs_tech_share_Retail_Trade" localSheetId="2">Europe!$C$83:$N$85</definedName>
-    <definedName name="ccs_tech_share_Hotels_and_Restaurants" localSheetId="2">Europe!$C$86:$N$88</definedName>
-    <definedName name="ccs_tech_share_Transport" localSheetId="2">Europe!$C$89:$N$91</definedName>
-    <definedName name="ccs_tech_share_Post_and_Telecomm" localSheetId="2">Europe!$C$92:$N$94</definedName>
-    <definedName name="ccs_tech_share_Offices" localSheetId="2">Europe!$C$95:$N$97</definedName>
-    <definedName name="ccs_tech_share_Education" localSheetId="2">Europe!$C$98:$N$100</definedName>
-    <definedName name="ccs_tech_share_Health_and_Social_work" localSheetId="2">Europe!$C$101:$N$103</definedName>
-    <definedName name="ccs_tech_share_Other_Community_Social_and_Personal_Services" localSheetId="2">Europe!$C$104:$N$106</definedName>
-    <definedName name="ccs_tech_share_Private_Households" localSheetId="2">Europe!$C$107:$N$109</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -10603,37 +10603,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201">
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>pre-combustion</t>
-        </is>
-      </c>
-      <c r="C201" t="n">
-        <v>0</v>
-      </c>
-      <c r="D201" t="n">
-        <v>0</v>
-      </c>
-      <c r="E201" t="n">
-        <v>0</v>
-      </c>
-      <c r="F201" t="n">
-        <v>0</v>
-      </c>
-      <c r="G201" t="n">
-        <v>0</v>
-      </c>
-      <c r="H201" t="n">
-        <v>0</v>
-      </c>
-      <c r="I201" t="n">
-        <v>0</v>
-      </c>
-      <c r="J201" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    <row r="201"/>
     <row r="202">
       <c r="B202" t="inlineStr">
         <is>
@@ -10805,7 +10775,6 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="206"/>
     <row r="207">
       <c r="A207" s="197" t="inlineStr">
         <is>
@@ -16021,37 +15990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108">
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>pre-combustion</t>
-        </is>
-      </c>
-      <c r="C108" t="n">
-        <v>0</v>
-      </c>
-      <c r="D108" t="n">
-        <v>0</v>
-      </c>
-      <c r="E108" t="n">
-        <v>0</v>
-      </c>
-      <c r="F108" t="n">
-        <v>0</v>
-      </c>
-      <c r="G108" t="n">
-        <v>0</v>
-      </c>
-      <c r="H108" t="n">
-        <v>0</v>
-      </c>
-      <c r="I108" t="n">
-        <v>0</v>
-      </c>
-      <c r="J108" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    <row r="108"/>
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
@@ -16223,7 +16162,6 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="113"/>
     <row r="114">
       <c r="A114" s="197" t="inlineStr">
         <is>
@@ -16987,43 +16925,43 @@
         </is>
       </c>
       <c r="D10" s="254" t="n">
-        <v>0</v>
+        <v>11997.68</v>
       </c>
       <c r="E10" s="254" t="n">
-        <v>0.00423265011842777</v>
+        <v>12000.1</v>
       </c>
       <c r="F10" s="254" t="n">
-        <v>0.00661813397651863</v>
+        <v>11605.9</v>
       </c>
       <c r="G10" s="254" t="n">
-        <v>0.0115558821163859</v>
+        <v>1491.67</v>
       </c>
       <c r="H10" s="254" t="n">
-        <v>0.121352943501787</v>
+        <v>1221.68</v>
       </c>
       <c r="I10" s="143" t="n">
-        <v>0</v>
+        <v>669.49</v>
       </c>
       <c r="J10" s="143" t="n">
-        <v>0</v>
+        <v>505.22</v>
       </c>
       <c r="K10" s="143" t="n">
-        <v>0</v>
+        <v>263.85</v>
       </c>
       <c r="L10" s="143" t="n">
-        <v>0</v>
+        <v>217.6</v>
       </c>
       <c r="M10" s="143" t="n">
-        <v>0</v>
+        <v>213.77</v>
       </c>
       <c r="N10" s="143" t="n">
-        <v>0</v>
+        <v>144.4</v>
       </c>
       <c r="O10" s="143" t="n">
-        <v>0</v>
+        <v>119.57</v>
       </c>
       <c r="P10" s="146" t="n">
-        <v>0</v>
+        <v>109.21</v>
       </c>
     </row>
     <row r="11">
@@ -17035,43 +16973,43 @@
         </is>
       </c>
       <c r="D11" s="254" t="n">
-        <v>0</v>
+        <v>11997.68</v>
       </c>
       <c r="E11" s="254" t="n">
-        <v>0.00423265011842777</v>
+        <v>12000.1</v>
       </c>
       <c r="F11" s="254" t="n">
-        <v>0.00661813397651863</v>
+        <v>11605.9</v>
       </c>
       <c r="G11" s="254" t="n">
-        <v>0.0115558821163859</v>
+        <v>10608.6</v>
       </c>
       <c r="H11" s="254" t="n">
-        <v>0.121352943501787</v>
+        <v>8441.5</v>
       </c>
       <c r="I11" s="147" t="n">
-        <v>0</v>
+        <v>8445.6</v>
       </c>
       <c r="J11" s="147" t="n">
-        <v>0</v>
+        <v>8663.4</v>
       </c>
       <c r="K11" s="147" t="n">
-        <v>0</v>
+        <v>9135.700000000001</v>
       </c>
       <c r="L11" s="147" t="n">
-        <v>0</v>
+        <v>8904.299999999999</v>
       </c>
       <c r="M11" s="147" t="n">
-        <v>0</v>
+        <v>9003.9</v>
       </c>
       <c r="N11" s="147" t="n">
-        <v>0</v>
+        <v>9465.200000000001</v>
       </c>
       <c r="O11" s="147" t="n">
-        <v>0</v>
+        <v>10581.6</v>
       </c>
       <c r="P11" s="150" t="n">
-        <v>0</v>
+        <v>11396.4</v>
       </c>
     </row>
     <row r="12">
@@ -17083,43 +17021,43 @@
         </is>
       </c>
       <c r="D12" s="254" t="n">
-        <v>0</v>
+        <v>11997.68</v>
       </c>
       <c r="E12" s="254" t="n">
-        <v>0.00423265011842777</v>
+        <v>12000.1</v>
       </c>
       <c r="F12" s="254" t="n">
-        <v>0.00661813397651863</v>
+        <v>11605.9</v>
       </c>
       <c r="G12" s="254" t="n">
-        <v>0.0115558821163859</v>
+        <v>22209.7</v>
       </c>
       <c r="H12" s="254" t="n">
-        <v>0.121352943501787</v>
+        <v>22873.5</v>
       </c>
       <c r="I12" s="147" t="n">
-        <v>0</v>
+        <v>23524.4</v>
       </c>
       <c r="J12" s="147" t="n">
-        <v>0</v>
+        <v>23833.3</v>
       </c>
       <c r="K12" s="147" t="n">
-        <v>0</v>
+        <v>23712.8</v>
       </c>
       <c r="L12" s="147" t="n">
-        <v>0</v>
+        <v>23725.3</v>
       </c>
       <c r="M12" s="147" t="n">
-        <v>0</v>
+        <v>23459.5</v>
       </c>
       <c r="N12" s="147" t="n">
-        <v>0</v>
+        <v>22934.6</v>
       </c>
       <c r="O12" s="147" t="n">
-        <v>0</v>
+        <v>21940.4</v>
       </c>
       <c r="P12" s="150" t="n">
-        <v>0</v>
+        <v>20799</v>
       </c>
     </row>
     <row r="13">
@@ -17131,43 +17069,43 @@
         </is>
       </c>
       <c r="D13" s="254" t="n">
-        <v>0</v>
+        <v>11997.68</v>
       </c>
       <c r="E13" s="254" t="n">
-        <v>0.00423265011842777</v>
+        <v>12000.1</v>
       </c>
       <c r="F13" s="254" t="n">
-        <v>0.00661813397651863</v>
+        <v>11605.9</v>
       </c>
       <c r="G13" s="254" t="n">
-        <v>0.0115558821163859</v>
+        <v>10634.4</v>
       </c>
       <c r="H13" s="254" t="n">
-        <v>0.121352943501787</v>
+        <v>11774.6</v>
       </c>
       <c r="I13" s="152" t="n">
-        <v>0</v>
+        <v>12414.8</v>
       </c>
       <c r="J13" s="152" t="n">
-        <v>0</v>
+        <v>12139.6</v>
       </c>
       <c r="K13" s="152" t="n">
-        <v>0</v>
+        <v>12490.8</v>
       </c>
       <c r="L13" s="152" t="n">
-        <v>0</v>
+        <v>11773.5</v>
       </c>
       <c r="M13" s="152" t="n">
-        <v>0</v>
+        <v>11840.9</v>
       </c>
       <c r="N13" s="152" t="n">
-        <v>0</v>
+        <v>11592.8</v>
       </c>
       <c r="O13" s="152" t="n">
-        <v>0</v>
+        <v>11093.2</v>
       </c>
       <c r="P13" s="155" t="n">
-        <v>0</v>
+        <v>10765.4</v>
       </c>
     </row>
     <row r="14">
@@ -17186,45 +17124,44 @@
           <t>RCP 2.6</t>
         </is>
       </c>
-      <c r="D14" s="254">
-        <f>0.000000552232907*1000000</f>
-        <v/>
+      <c r="D14" s="254" t="n">
+        <v>5520.77</v>
       </c>
       <c r="E14" s="254" t="n">
-        <v>1.434020062</v>
+        <v>5538</v>
       </c>
       <c r="F14" s="254" t="n">
-        <v>1.744082373</v>
+        <v>6341</v>
       </c>
       <c r="G14" s="254" t="n">
-        <v>1.851693432</v>
+        <v>6623.1</v>
       </c>
       <c r="H14" s="254" t="n">
-        <v>1.774427471</v>
+        <v>2244.2</v>
       </c>
       <c r="I14" s="143" t="n">
-        <v>0</v>
+        <v>1952.3</v>
       </c>
       <c r="J14" s="143" t="n">
-        <v>0</v>
+        <v>1567.6</v>
       </c>
       <c r="K14" s="143" t="n">
-        <v>0</v>
+        <v>632.2</v>
       </c>
       <c r="L14" s="143" t="n">
-        <v>0</v>
+        <v>498.5</v>
       </c>
       <c r="M14" s="143" t="n">
-        <v>0</v>
+        <v>418.3</v>
       </c>
       <c r="N14" s="143" t="n">
-        <v>0</v>
+        <v>315.8</v>
       </c>
       <c r="O14" s="143" t="n">
-        <v>0</v>
+        <v>185.2</v>
       </c>
       <c r="P14" s="146" t="n">
-        <v>0</v>
+        <v>44.2</v>
       </c>
     </row>
     <row r="15">
@@ -17235,45 +17172,44 @@
           <t>RCP 4.5</t>
         </is>
       </c>
-      <c r="D15" s="254">
-        <f>0.000000552232907*1000000</f>
-        <v/>
+      <c r="D15" s="254" t="n">
+        <v>5520.77</v>
       </c>
       <c r="E15" s="254" t="n">
-        <v>1.434020062</v>
+        <v>5538</v>
       </c>
       <c r="F15" s="254" t="n">
-        <v>1.744082373</v>
+        <v>6341</v>
       </c>
       <c r="G15" s="254" t="n">
-        <v>1.851693432</v>
+        <v>5655.4</v>
       </c>
       <c r="H15" s="254" t="n">
-        <v>1.774427471</v>
+        <v>2502.7</v>
       </c>
       <c r="I15" s="147" t="n">
-        <v>0</v>
+        <v>2910.9</v>
       </c>
       <c r="J15" s="147" t="n">
-        <v>0</v>
+        <v>3337.1</v>
       </c>
       <c r="K15" s="147" t="n">
-        <v>0</v>
+        <v>3781.6</v>
       </c>
       <c r="L15" s="147" t="n">
-        <v>0</v>
+        <v>4293</v>
       </c>
       <c r="M15" s="147" t="n">
-        <v>0</v>
+        <v>4894.8</v>
       </c>
       <c r="N15" s="147" t="n">
-        <v>0</v>
+        <v>5586.9</v>
       </c>
       <c r="O15" s="147" t="n">
-        <v>0</v>
+        <v>6010.6</v>
       </c>
       <c r="P15" s="150" t="n">
-        <v>0</v>
+        <v>6434.3</v>
       </c>
     </row>
     <row r="16">
@@ -17284,45 +17220,44 @@
           <t>RCP 6.0</t>
         </is>
       </c>
-      <c r="D16" s="254">
-        <f>0.000000552232907*1000000</f>
-        <v/>
+      <c r="D16" s="254" t="n">
+        <v>5520.77</v>
       </c>
       <c r="E16" s="254" t="n">
-        <v>1.434020062</v>
+        <v>5538</v>
       </c>
       <c r="F16" s="254" t="n">
-        <v>1.744082373</v>
+        <v>6341</v>
       </c>
       <c r="G16" s="254" t="n">
-        <v>1.851693432</v>
+        <v>7770.3</v>
       </c>
       <c r="H16" s="254" t="n">
-        <v>1.774427471</v>
+        <v>9425.4</v>
       </c>
       <c r="I16" s="147" t="n">
-        <v>0</v>
+        <v>9602.5</v>
       </c>
       <c r="J16" s="147" t="n">
-        <v>0</v>
+        <v>9687.299999999999</v>
       </c>
       <c r="K16" s="147" t="n">
-        <v>0</v>
+        <v>9779.5</v>
       </c>
       <c r="L16" s="147" t="n">
-        <v>0</v>
+        <v>9928</v>
       </c>
       <c r="M16" s="147" t="n">
-        <v>0</v>
+        <v>10082.8</v>
       </c>
       <c r="N16" s="147" t="n">
-        <v>0</v>
+        <v>9996.1</v>
       </c>
       <c r="O16" s="147" t="n">
-        <v>0</v>
+        <v>9874.9</v>
       </c>
       <c r="P16" s="150" t="n">
-        <v>0</v>
+        <v>9497.1</v>
       </c>
     </row>
     <row r="17">
@@ -17333,45 +17268,44 @@
           <t>RCP 8.5</t>
         </is>
       </c>
-      <c r="D17" s="254">
-        <f>0.000000552232907*1000000</f>
-        <v/>
+      <c r="D17" s="254" t="n">
+        <v>5520.77</v>
       </c>
       <c r="E17" s="254" t="n">
-        <v>1.434020062</v>
+        <v>5538</v>
       </c>
       <c r="F17" s="254" t="n">
-        <v>1.744082373</v>
+        <v>6341</v>
       </c>
       <c r="G17" s="254" t="n">
-        <v>1.851693432</v>
+        <v>7044.3</v>
       </c>
       <c r="H17" s="254" t="n">
-        <v>1.774427471</v>
+        <v>8081.2</v>
       </c>
       <c r="I17" s="158" t="n">
-        <v>0</v>
+        <v>9988.299999999999</v>
       </c>
       <c r="J17" s="158" t="n">
-        <v>0</v>
+        <v>11260.3</v>
       </c>
       <c r="K17" s="158" t="n">
-        <v>0</v>
+        <v>11965.3</v>
       </c>
       <c r="L17" s="158" t="n">
-        <v>0</v>
+        <v>14059.7</v>
       </c>
       <c r="M17" s="158" t="n">
-        <v>0</v>
+        <v>13492</v>
       </c>
       <c r="N17" s="158" t="n">
-        <v>0</v>
+        <v>14875.8</v>
       </c>
       <c r="O17" s="158" t="n">
-        <v>0</v>
+        <v>16052.7</v>
       </c>
       <c r="P17" s="159" t="n">
-        <v>0</v>
+        <v>16922.3</v>
       </c>
     </row>
     <row r="18">
@@ -17413,43 +17347,43 @@
         </is>
       </c>
       <c r="D19" s="148" t="n">
-        <v>0</v>
+        <v>1010</v>
       </c>
       <c r="E19" s="148" t="n">
-        <v>0</v>
+        <v>75039</v>
       </c>
       <c r="F19" s="149" t="n">
-        <v>0</v>
+        <v>120933</v>
       </c>
       <c r="G19" s="148" t="n">
-        <v>0</v>
+        <v>157043</v>
       </c>
       <c r="H19" s="148" t="n">
-        <v>0</v>
+        <v>173879</v>
       </c>
       <c r="I19" s="148" t="n">
-        <v>0</v>
+        <v>194186</v>
       </c>
       <c r="J19" s="148" t="n">
-        <v>0</v>
+        <v>212829</v>
       </c>
       <c r="K19" s="148" t="n">
-        <v>0</v>
+        <v>198351</v>
       </c>
       <c r="L19" s="148" t="n">
-        <v>0</v>
+        <v>226357</v>
       </c>
       <c r="M19" s="148" t="n">
-        <v>0</v>
+        <v>255846</v>
       </c>
       <c r="N19" s="148" t="n">
-        <v>0</v>
+        <v>265700</v>
       </c>
       <c r="O19" s="148" t="n">
-        <v>0</v>
+        <v>256848</v>
       </c>
       <c r="P19" s="163" t="n">
-        <v>0</v>
+        <v>235392</v>
       </c>
     </row>
     <row r="20">
@@ -17461,43 +17395,43 @@
         </is>
       </c>
       <c r="D20" s="148" t="n">
-        <v>0</v>
+        <v>1010</v>
       </c>
       <c r="E20" s="148" t="n">
-        <v>0</v>
+        <v>75039</v>
       </c>
       <c r="F20" s="149" t="n">
-        <v>0</v>
+        <v>120933</v>
       </c>
       <c r="G20" s="148" t="n">
-        <v>0</v>
+        <v>142731</v>
       </c>
       <c r="H20" s="148" t="n">
-        <v>0</v>
+        <v>189436</v>
       </c>
       <c r="I20" s="148" t="n">
-        <v>0</v>
+        <v>208276</v>
       </c>
       <c r="J20" s="148" t="n">
-        <v>0</v>
+        <v>229429</v>
       </c>
       <c r="K20" s="148" t="n">
-        <v>0</v>
+        <v>252971</v>
       </c>
       <c r="L20" s="148" t="n">
-        <v>0</v>
+        <v>243443</v>
       </c>
       <c r="M20" s="148" t="n">
-        <v>0</v>
+        <v>258052</v>
       </c>
       <c r="N20" s="148" t="n">
-        <v>0</v>
+        <v>300616</v>
       </c>
       <c r="O20" s="148" t="n">
-        <v>0</v>
+        <v>353004</v>
       </c>
       <c r="P20" s="163" t="n">
-        <v>0</v>
+        <v>409075</v>
       </c>
     </row>
     <row r="21">
@@ -17509,43 +17443,43 @@
         </is>
       </c>
       <c r="D21" s="148" t="n">
-        <v>0</v>
+        <v>1010</v>
       </c>
       <c r="E21" s="148" t="n">
-        <v>0</v>
+        <v>75039</v>
       </c>
       <c r="F21" s="149" t="n">
-        <v>0</v>
+        <v>120933</v>
       </c>
       <c r="G21" s="148" t="n">
-        <v>0</v>
+        <v>146301</v>
       </c>
       <c r="H21" s="148" t="n">
-        <v>0</v>
+        <v>153891</v>
       </c>
       <c r="I21" s="148" t="n">
-        <v>0</v>
+        <v>159119</v>
       </c>
       <c r="J21" s="148" t="n">
-        <v>0</v>
+        <v>163629</v>
       </c>
       <c r="K21" s="148" t="n">
-        <v>0</v>
+        <v>167105</v>
       </c>
       <c r="L21" s="148" t="n">
-        <v>0</v>
+        <v>171969</v>
       </c>
       <c r="M21" s="148" t="n">
-        <v>0</v>
+        <v>175922</v>
       </c>
       <c r="N21" s="148" t="n">
-        <v>0</v>
+        <v>177072</v>
       </c>
       <c r="O21" s="148" t="n">
-        <v>0</v>
+        <v>174566</v>
       </c>
       <c r="P21" s="163" t="n">
-        <v>0</v>
+        <v>170500</v>
       </c>
     </row>
     <row r="22">
@@ -17557,43 +17491,43 @@
         </is>
       </c>
       <c r="D22" s="148" t="n">
-        <v>0</v>
+        <v>1010</v>
       </c>
       <c r="E22" s="148" t="n">
-        <v>0</v>
+        <v>75039</v>
       </c>
       <c r="F22" s="149" t="n">
-        <v>0</v>
+        <v>120933</v>
       </c>
       <c r="G22" s="148" t="n">
-        <v>0</v>
+        <v>152513</v>
       </c>
       <c r="H22" s="148" t="n">
-        <v>0</v>
+        <v>265080</v>
       </c>
       <c r="I22" s="148" t="n">
-        <v>0</v>
+        <v>333876</v>
       </c>
       <c r="J22" s="148" t="n">
-        <v>0</v>
+        <v>406963</v>
       </c>
       <c r="K22" s="148" t="n">
-        <v>0</v>
+        <v>464903</v>
       </c>
       <c r="L22" s="148" t="n">
-        <v>0</v>
+        <v>508058</v>
       </c>
       <c r="M22" s="148" t="n">
-        <v>0</v>
+        <v>554713</v>
       </c>
       <c r="N22" s="148" t="n">
-        <v>0</v>
+        <v>605051</v>
       </c>
       <c r="O22" s="148" t="n">
-        <v>0</v>
+        <v>653132</v>
       </c>
       <c r="P22" s="163" t="n">
-        <v>0</v>
+        <v>703459</v>
       </c>
     </row>
     <row r="23">
@@ -17613,37 +17547,37 @@
         </is>
       </c>
       <c r="D23" s="148" t="n">
-        <v>0</v>
+        <v>6622</v>
       </c>
       <c r="E23" s="148" t="n">
-        <v>0</v>
+        <v>10395</v>
       </c>
       <c r="F23" s="148" t="n">
-        <v>0</v>
+        <v>10812</v>
       </c>
       <c r="G23" s="148" t="n">
-        <v>0</v>
+        <v>9522</v>
       </c>
       <c r="H23" s="148" t="n">
-        <v>0</v>
+        <v>1152</v>
       </c>
       <c r="I23" s="148" t="n">
-        <v>0</v>
+        <v>691</v>
       </c>
       <c r="J23" s="148" t="n">
-        <v>0</v>
+        <v>413</v>
       </c>
       <c r="K23" s="148" t="n">
-        <v>0</v>
+        <v>246</v>
       </c>
       <c r="L23" s="148" t="n">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="M23" s="148" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="N23" s="148" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="O23" s="148" t="n">
         <v>0</v>
@@ -17661,37 +17595,37 @@
         </is>
       </c>
       <c r="D24" s="148" t="n">
-        <v>0</v>
+        <v>6622</v>
       </c>
       <c r="E24" s="148" t="n">
-        <v>0</v>
+        <v>10395</v>
       </c>
       <c r="F24" s="148" t="n">
-        <v>0</v>
+        <v>10812</v>
       </c>
       <c r="G24" s="148" t="n">
-        <v>0</v>
+        <v>9522</v>
       </c>
       <c r="H24" s="148" t="n">
-        <v>0</v>
+        <v>1152</v>
       </c>
       <c r="I24" s="148" t="n">
-        <v>0</v>
+        <v>691</v>
       </c>
       <c r="J24" s="148" t="n">
-        <v>0</v>
+        <v>413</v>
       </c>
       <c r="K24" s="148" t="n">
-        <v>0</v>
+        <v>246</v>
       </c>
       <c r="L24" s="148" t="n">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="M24" s="148" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="N24" s="148" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="O24" s="148" t="n">
         <v>0</v>
@@ -17709,37 +17643,37 @@
         </is>
       </c>
       <c r="D25" s="148" t="n">
-        <v>0</v>
+        <v>6622</v>
       </c>
       <c r="E25" s="148" t="n">
-        <v>0</v>
+        <v>10395</v>
       </c>
       <c r="F25" s="148" t="n">
-        <v>0</v>
+        <v>10812</v>
       </c>
       <c r="G25" s="148" t="n">
-        <v>0</v>
+        <v>9522</v>
       </c>
       <c r="H25" s="148" t="n">
-        <v>0</v>
+        <v>1152</v>
       </c>
       <c r="I25" s="148" t="n">
-        <v>0</v>
+        <v>691</v>
       </c>
       <c r="J25" s="148" t="n">
-        <v>0</v>
+        <v>413</v>
       </c>
       <c r="K25" s="148" t="n">
-        <v>0</v>
+        <v>246</v>
       </c>
       <c r="L25" s="148" t="n">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="M25" s="148" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="N25" s="148" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="O25" s="148" t="n">
         <v>0</v>
@@ -17757,37 +17691,37 @@
         </is>
       </c>
       <c r="D26" s="148" t="n">
-        <v>0</v>
+        <v>6622</v>
       </c>
       <c r="E26" s="148" t="n">
-        <v>0</v>
+        <v>10395</v>
       </c>
       <c r="F26" s="148" t="n">
-        <v>0</v>
+        <v>10812</v>
       </c>
       <c r="G26" s="148" t="n">
-        <v>0</v>
+        <v>9522</v>
       </c>
       <c r="H26" s="148" t="n">
-        <v>0</v>
+        <v>1152</v>
       </c>
       <c r="I26" s="148" t="n">
-        <v>0</v>
+        <v>691</v>
       </c>
       <c r="J26" s="148" t="n">
-        <v>0</v>
+        <v>413</v>
       </c>
       <c r="K26" s="148" t="n">
-        <v>0</v>
+        <v>246</v>
       </c>
       <c r="L26" s="148" t="n">
-        <v>0</v>
+        <v>138</v>
       </c>
       <c r="M26" s="148" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="N26" s="148" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="O26" s="148" t="n">
         <v>0</v>
@@ -17816,40 +17750,40 @@
         <v>0</v>
       </c>
       <c r="E27" s="148" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="F27" s="149" t="n">
-        <v>0</v>
+        <v>10994</v>
       </c>
       <c r="G27" s="148" t="n">
-        <v>0</v>
+        <v>17942</v>
       </c>
       <c r="H27" s="148" t="n">
-        <v>0</v>
+        <v>60642</v>
       </c>
       <c r="I27" s="148" t="n">
-        <v>0</v>
+        <v>72035</v>
       </c>
       <c r="J27" s="148" t="n">
-        <v>0</v>
+        <v>80712</v>
       </c>
       <c r="K27" s="148" t="n">
-        <v>0</v>
+        <v>74607</v>
       </c>
       <c r="L27" s="148" t="n">
-        <v>0</v>
+        <v>84086</v>
       </c>
       <c r="M27" s="148" t="n">
-        <v>0</v>
+        <v>93880</v>
       </c>
       <c r="N27" s="148" t="n">
-        <v>0</v>
+        <v>96271</v>
       </c>
       <c r="O27" s="148" t="n">
-        <v>0</v>
+        <v>91204</v>
       </c>
       <c r="P27" s="163" t="n">
-        <v>0</v>
+        <v>81227</v>
       </c>
     </row>
     <row r="28">
@@ -17864,40 +17798,40 @@
         <v>0</v>
       </c>
       <c r="E28" s="148" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="F28" s="149" t="n">
-        <v>0</v>
+        <v>10994</v>
       </c>
       <c r="G28" s="148" t="n">
-        <v>0</v>
+        <v>17942</v>
       </c>
       <c r="H28" s="148" t="n">
-        <v>0</v>
+        <v>60642</v>
       </c>
       <c r="I28" s="148" t="n">
-        <v>0</v>
+        <v>72035</v>
       </c>
       <c r="J28" s="148" t="n">
-        <v>0</v>
+        <v>80712</v>
       </c>
       <c r="K28" s="148" t="n">
-        <v>0</v>
+        <v>74607</v>
       </c>
       <c r="L28" s="148" t="n">
-        <v>0</v>
+        <v>84086</v>
       </c>
       <c r="M28" s="148" t="n">
-        <v>0</v>
+        <v>93880</v>
       </c>
       <c r="N28" s="148" t="n">
-        <v>0</v>
+        <v>96271</v>
       </c>
       <c r="O28" s="148" t="n">
-        <v>0</v>
+        <v>91204</v>
       </c>
       <c r="P28" s="163" t="n">
-        <v>0</v>
+        <v>81227</v>
       </c>
     </row>
     <row r="29">
@@ -17912,40 +17846,40 @@
         <v>0</v>
       </c>
       <c r="E29" s="148" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="F29" s="149" t="n">
-        <v>0</v>
+        <v>10994</v>
       </c>
       <c r="G29" s="148" t="n">
-        <v>0</v>
+        <v>17942</v>
       </c>
       <c r="H29" s="148" t="n">
-        <v>0</v>
+        <v>60642</v>
       </c>
       <c r="I29" s="148" t="n">
-        <v>0</v>
+        <v>72035</v>
       </c>
       <c r="J29" s="148" t="n">
-        <v>0</v>
+        <v>80712</v>
       </c>
       <c r="K29" s="148" t="n">
-        <v>0</v>
+        <v>74607</v>
       </c>
       <c r="L29" s="148" t="n">
-        <v>0</v>
+        <v>84086</v>
       </c>
       <c r="M29" s="148" t="n">
-        <v>0</v>
+        <v>93880</v>
       </c>
       <c r="N29" s="148" t="n">
-        <v>0</v>
+        <v>96271</v>
       </c>
       <c r="O29" s="148" t="n">
-        <v>0</v>
+        <v>91204</v>
       </c>
       <c r="P29" s="163" t="n">
-        <v>0</v>
+        <v>81227</v>
       </c>
     </row>
     <row r="30">
@@ -17960,40 +17894,40 @@
         <v>0</v>
       </c>
       <c r="E30" s="148" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="F30" s="149" t="n">
-        <v>0</v>
+        <v>10994</v>
       </c>
       <c r="G30" s="148" t="n">
-        <v>0</v>
+        <v>17942</v>
       </c>
       <c r="H30" s="148" t="n">
-        <v>0</v>
+        <v>60642</v>
       </c>
       <c r="I30" s="148" t="n">
-        <v>0</v>
+        <v>72035</v>
       </c>
       <c r="J30" s="148" t="n">
-        <v>0</v>
+        <v>80712</v>
       </c>
       <c r="K30" s="148" t="n">
-        <v>0</v>
+        <v>74607</v>
       </c>
       <c r="L30" s="148" t="n">
-        <v>0</v>
+        <v>84086</v>
       </c>
       <c r="M30" s="148" t="n">
-        <v>0</v>
+        <v>93880</v>
       </c>
       <c r="N30" s="148" t="n">
-        <v>0</v>
+        <v>96271</v>
       </c>
       <c r="O30" s="148" t="n">
-        <v>0</v>
+        <v>91204</v>
       </c>
       <c r="P30" s="163" t="n">
-        <v>0</v>
+        <v>81227</v>
       </c>
     </row>
     <row r="31">
@@ -18013,43 +17947,43 @@
         </is>
       </c>
       <c r="D31" s="165" t="n">
-        <v>0</v>
+        <v>186</v>
       </c>
       <c r="E31" s="165" t="n">
-        <v>0</v>
+        <v>8538</v>
       </c>
       <c r="F31" s="166" t="n">
-        <v>0</v>
+        <v>13759</v>
       </c>
       <c r="G31" s="166" t="n">
-        <v>0</v>
+        <v>26279</v>
       </c>
       <c r="H31" s="166" t="n">
-        <v>0</v>
+        <v>89349</v>
       </c>
       <c r="I31" s="166" t="n">
-        <v>0</v>
+        <v>108899</v>
       </c>
       <c r="J31" s="166" t="n">
-        <v>0</v>
+        <v>124961</v>
       </c>
       <c r="K31" s="166" t="n">
-        <v>0</v>
+        <v>119137</v>
       </c>
       <c r="L31" s="166" t="n">
-        <v>0</v>
+        <v>138797</v>
       </c>
       <c r="M31" s="166" t="n">
-        <v>0</v>
+        <v>159182</v>
       </c>
       <c r="N31" s="166" t="n">
-        <v>0</v>
+        <v>166569</v>
       </c>
       <c r="O31" s="166" t="n">
-        <v>0</v>
+        <v>161556</v>
       </c>
       <c r="P31" s="167" t="n">
-        <v>0</v>
+        <v>148214</v>
       </c>
     </row>
     <row r="32">
@@ -18061,43 +17995,43 @@
         </is>
       </c>
       <c r="D32" s="165" t="n">
-        <v>0</v>
+        <v>186</v>
       </c>
       <c r="E32" s="165" t="n">
-        <v>0</v>
+        <v>8538</v>
       </c>
       <c r="F32" s="166" t="n">
-        <v>0</v>
+        <v>13759</v>
       </c>
       <c r="G32" s="166" t="n">
-        <v>0</v>
+        <v>17127</v>
       </c>
       <c r="H32" s="166" t="n">
-        <v>0</v>
+        <v>31282</v>
       </c>
       <c r="I32" s="166" t="n">
-        <v>0</v>
+        <v>31762</v>
       </c>
       <c r="J32" s="166" t="n">
-        <v>0</v>
+        <v>31380</v>
       </c>
       <c r="K32" s="166" t="n">
-        <v>0</v>
+        <v>30710</v>
       </c>
       <c r="L32" s="166" t="n">
-        <v>0</v>
+        <v>26222</v>
       </c>
       <c r="M32" s="166" t="n">
-        <v>0</v>
+        <v>23990</v>
       </c>
       <c r="N32" s="166" t="n">
-        <v>0</v>
+        <v>23536</v>
       </c>
       <c r="O32" s="166" t="n">
-        <v>0</v>
+        <v>23520</v>
       </c>
       <c r="P32" s="167" t="n">
-        <v>0</v>
+        <v>23006</v>
       </c>
     </row>
     <row r="33">
@@ -18109,43 +18043,43 @@
         </is>
       </c>
       <c r="D33" s="165" t="n">
-        <v>0</v>
+        <v>186</v>
       </c>
       <c r="E33" s="165" t="n">
-        <v>0</v>
+        <v>8538</v>
       </c>
       <c r="F33" s="166" t="n">
-        <v>0</v>
+        <v>13759</v>
       </c>
       <c r="G33" s="166" t="n">
-        <v>0</v>
+        <v>8121</v>
       </c>
       <c r="H33" s="166" t="n">
-        <v>0</v>
+        <v>8889</v>
       </c>
       <c r="I33" s="166" t="n">
-        <v>0</v>
+        <v>9418</v>
       </c>
       <c r="J33" s="166" t="n">
-        <v>0</v>
+        <v>10006</v>
       </c>
       <c r="K33" s="166" t="n">
-        <v>0</v>
+        <v>10385</v>
       </c>
       <c r="L33" s="166" t="n">
-        <v>0</v>
+        <v>10938</v>
       </c>
       <c r="M33" s="166" t="n">
-        <v>0</v>
+        <v>11420</v>
       </c>
       <c r="N33" s="166" t="n">
-        <v>0</v>
+        <v>11739</v>
       </c>
       <c r="O33" s="166" t="n">
-        <v>0</v>
+        <v>11779</v>
       </c>
       <c r="P33" s="167" t="n">
-        <v>0</v>
+        <v>11699</v>
       </c>
     </row>
     <row r="34">
@@ -18157,43 +18091,43 @@
         </is>
       </c>
       <c r="D34" s="165" t="n">
-        <v>0</v>
+        <v>186</v>
       </c>
       <c r="E34" s="165" t="n">
-        <v>0</v>
+        <v>8538</v>
       </c>
       <c r="F34" s="166" t="n">
-        <v>0</v>
+        <v>13759</v>
       </c>
       <c r="G34" s="166" t="n">
-        <v>0</v>
+        <v>34598</v>
       </c>
       <c r="H34" s="166" t="n">
-        <v>0</v>
+        <v>66696</v>
       </c>
       <c r="I34" s="166" t="n">
-        <v>0</v>
+        <v>78956</v>
       </c>
       <c r="J34" s="166" t="n">
-        <v>0</v>
+        <v>100250</v>
       </c>
       <c r="K34" s="166" t="n">
-        <v>0</v>
+        <v>116135</v>
       </c>
       <c r="L34" s="166" t="n">
-        <v>0</v>
+        <v>128080</v>
       </c>
       <c r="M34" s="166" t="n">
-        <v>0</v>
+        <v>140714</v>
       </c>
       <c r="N34" s="166" t="n">
-        <v>0</v>
+        <v>144726</v>
       </c>
       <c r="O34" s="166" t="n">
-        <v>0</v>
+        <v>147547</v>
       </c>
       <c r="P34" s="167" t="n">
-        <v>0</v>
+        <v>148304</v>
       </c>
     </row>
     <row r="35">
@@ -18213,43 +18147,43 @@
         </is>
       </c>
       <c r="D35" s="148" t="n">
-        <v>0</v>
+        <v>889</v>
       </c>
       <c r="E35" s="148" t="n">
-        <v>0</v>
+        <v>6234</v>
       </c>
       <c r="F35" s="149" t="n">
-        <v>0</v>
+        <v>12448</v>
       </c>
       <c r="G35" s="149" t="n">
-        <v>0</v>
+        <v>21616</v>
       </c>
       <c r="H35" s="149" t="n">
-        <v>0</v>
+        <v>64374</v>
       </c>
       <c r="I35" s="149" t="n">
-        <v>0</v>
+        <v>75555</v>
       </c>
       <c r="J35" s="149" t="n">
-        <v>0</v>
+        <v>83724</v>
       </c>
       <c r="K35" s="149" t="n">
-        <v>0</v>
+        <v>77089</v>
       </c>
       <c r="L35" s="149" t="n">
-        <v>0</v>
+        <v>86593</v>
       </c>
       <c r="M35" s="149" t="n">
-        <v>0</v>
+        <v>95507</v>
       </c>
       <c r="N35" s="149" t="n">
-        <v>0</v>
+        <v>95810</v>
       </c>
       <c r="O35" s="149" t="n">
-        <v>0</v>
+        <v>88763</v>
       </c>
       <c r="P35" s="168" t="n">
-        <v>0</v>
+        <v>77457</v>
       </c>
     </row>
     <row r="36">
@@ -18261,43 +18195,43 @@
         </is>
       </c>
       <c r="D36" s="148" t="n">
-        <v>0</v>
+        <v>889</v>
       </c>
       <c r="E36" s="148" t="n">
-        <v>0</v>
+        <v>6234</v>
       </c>
       <c r="F36" s="149" t="n">
-        <v>0</v>
+        <v>12448</v>
       </c>
       <c r="G36" s="149" t="n">
-        <v>0</v>
+        <v>14163</v>
       </c>
       <c r="H36" s="149" t="n">
-        <v>0</v>
+        <v>17666</v>
       </c>
       <c r="I36" s="149" t="n">
-        <v>0</v>
+        <v>20459</v>
       </c>
       <c r="J36" s="149" t="n">
-        <v>0</v>
+        <v>23292</v>
       </c>
       <c r="K36" s="149" t="n">
-        <v>0</v>
+        <v>26118</v>
       </c>
       <c r="L36" s="149" t="n">
-        <v>0</v>
+        <v>25539</v>
       </c>
       <c r="M36" s="149" t="n">
-        <v>0</v>
+        <v>28046</v>
       </c>
       <c r="N36" s="149" t="n">
-        <v>0</v>
+        <v>33790</v>
       </c>
       <c r="O36" s="149" t="n">
-        <v>0</v>
+        <v>39928</v>
       </c>
       <c r="P36" s="168" t="n">
-        <v>0</v>
+        <v>46270</v>
       </c>
     </row>
     <row r="37">
@@ -18309,43 +18243,43 @@
         </is>
       </c>
       <c r="D37" s="148" t="n">
-        <v>0</v>
+        <v>889</v>
       </c>
       <c r="E37" s="148" t="n">
-        <v>0</v>
+        <v>6234</v>
       </c>
       <c r="F37" s="149" t="n">
-        <v>0</v>
+        <v>12448</v>
       </c>
       <c r="G37" s="149" t="n">
-        <v>0</v>
+        <v>4514</v>
       </c>
       <c r="H37" s="149" t="n">
-        <v>0</v>
+        <v>5554</v>
       </c>
       <c r="I37" s="149" t="n">
-        <v>0</v>
+        <v>6059</v>
       </c>
       <c r="J37" s="149" t="n">
-        <v>0</v>
+        <v>6639</v>
       </c>
       <c r="K37" s="149" t="n">
-        <v>0</v>
+        <v>7119</v>
       </c>
       <c r="L37" s="149" t="n">
-        <v>0</v>
+        <v>7758</v>
       </c>
       <c r="M37" s="149" t="n">
-        <v>0</v>
+        <v>8342</v>
       </c>
       <c r="N37" s="149" t="n">
-        <v>0</v>
+        <v>8768</v>
       </c>
       <c r="O37" s="149" t="n">
-        <v>0</v>
+        <v>8999</v>
       </c>
       <c r="P37" s="168" t="n">
-        <v>0</v>
+        <v>9099</v>
       </c>
     </row>
     <row r="38">
@@ -18357,43 +18291,43 @@
         </is>
       </c>
       <c r="D38" s="148" t="n">
-        <v>0</v>
+        <v>889</v>
       </c>
       <c r="E38" s="148" t="n">
-        <v>0</v>
+        <v>6234</v>
       </c>
       <c r="F38" s="149" t="n">
-        <v>0</v>
+        <v>12448</v>
       </c>
       <c r="G38" s="149" t="n">
-        <v>0</v>
+        <v>26537</v>
       </c>
       <c r="H38" s="149" t="n">
-        <v>0</v>
+        <v>35067</v>
       </c>
       <c r="I38" s="149" t="n">
-        <v>0</v>
+        <v>38184</v>
       </c>
       <c r="J38" s="149" t="n">
-        <v>0</v>
+        <v>45837</v>
       </c>
       <c r="K38" s="149" t="n">
-        <v>0</v>
+        <v>50207</v>
       </c>
       <c r="L38" s="149" t="n">
-        <v>0</v>
+        <v>52424</v>
       </c>
       <c r="M38" s="149" t="n">
-        <v>0</v>
+        <v>54619</v>
       </c>
       <c r="N38" s="149" t="n">
-        <v>0</v>
+        <v>52707</v>
       </c>
       <c r="O38" s="149" t="n">
-        <v>0</v>
+        <v>50177</v>
       </c>
       <c r="P38" s="168" t="n">
-        <v>0</v>
+        <v>46842</v>
       </c>
     </row>
     <row r="39">
@@ -18413,16 +18347,16 @@
         </is>
       </c>
       <c r="D39" s="148" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E39" s="148" t="n">
-        <v>0</v>
+        <v>15200</v>
       </c>
       <c r="F39" s="149" t="n">
-        <v>0</v>
+        <v>23010</v>
       </c>
       <c r="G39" s="148" t="n">
-        <v>0</v>
+        <v>34530</v>
       </c>
       <c r="H39" s="148" t="n">
         <v>0</v>
@@ -18461,16 +18395,16 @@
         </is>
       </c>
       <c r="D40" s="169" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E40" s="169" t="n">
-        <v>0</v>
+        <v>15200</v>
       </c>
       <c r="F40" s="149" t="n">
-        <v>0</v>
+        <v>23010</v>
       </c>
       <c r="G40" s="148" t="n">
-        <v>0</v>
+        <v>34530</v>
       </c>
       <c r="H40" s="148" t="n">
         <v>0</v>
@@ -18509,16 +18443,16 @@
         </is>
       </c>
       <c r="D41" s="148" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E41" s="148" t="n">
-        <v>0</v>
+        <v>15200</v>
       </c>
       <c r="F41" s="149" t="n">
-        <v>0</v>
+        <v>23010</v>
       </c>
       <c r="G41" s="148" t="n">
-        <v>0</v>
+        <v>34530</v>
       </c>
       <c r="H41" s="148" t="n">
         <v>0</v>
@@ -18557,16 +18491,16 @@
         </is>
       </c>
       <c r="D42" s="148" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E42" s="148" t="n">
-        <v>0</v>
+        <v>15200</v>
       </c>
       <c r="F42" s="149" t="n">
-        <v>0</v>
+        <v>23010</v>
       </c>
       <c r="G42" s="148" t="n">
-        <v>0</v>
+        <v>34530</v>
       </c>
       <c r="H42" s="148" t="n">
         <v>0</v>
@@ -18616,40 +18550,40 @@
         <v>0</v>
       </c>
       <c r="E43" s="148" t="n">
-        <v>0</v>
+        <v>1951</v>
       </c>
       <c r="F43" s="149" t="n">
-        <v>0</v>
+        <v>4890</v>
       </c>
       <c r="G43" s="149" t="n">
-        <v>0</v>
+        <v>8979</v>
       </c>
       <c r="H43" s="149" t="n">
-        <v>0</v>
+        <v>1608</v>
       </c>
       <c r="I43" s="149" t="n">
-        <v>0</v>
+        <v>795</v>
       </c>
       <c r="J43" s="149" t="n">
-        <v>0</v>
+        <v>886</v>
       </c>
       <c r="K43" s="149" t="n">
-        <v>0</v>
+        <v>296</v>
       </c>
       <c r="L43" s="149" t="n">
-        <v>0</v>
+        <v>142</v>
       </c>
       <c r="M43" s="149" t="n">
-        <v>0</v>
+        <v>132</v>
       </c>
       <c r="N43" s="149" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="O43" s="149" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="P43" s="168" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
     </row>
     <row r="44">
@@ -18664,40 +18598,40 @@
         <v>0</v>
       </c>
       <c r="E44" s="148" t="n">
-        <v>0</v>
+        <v>1951</v>
       </c>
       <c r="F44" s="149" t="n">
-        <v>0</v>
+        <v>4890</v>
       </c>
       <c r="G44" s="149" t="n">
-        <v>0</v>
+        <v>6212</v>
       </c>
       <c r="H44" s="149" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="I44" s="149" t="n">
-        <v>0</v>
+        <v>258</v>
       </c>
       <c r="J44" s="149" t="n">
-        <v>0</v>
+        <v>257</v>
       </c>
       <c r="K44" s="149" t="n">
-        <v>0</v>
+        <v>89</v>
       </c>
       <c r="L44" s="149" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="M44" s="149" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="N44" s="149" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="O44" s="149" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="P44" s="168" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="45">
@@ -18712,40 +18646,40 @@
         <v>0</v>
       </c>
       <c r="E45" s="148" t="n">
-        <v>0</v>
+        <v>1951</v>
       </c>
       <c r="F45" s="149" t="n">
-        <v>0</v>
+        <v>4890</v>
       </c>
       <c r="G45" s="149" t="n">
-        <v>0</v>
+        <v>8820</v>
       </c>
       <c r="H45" s="149" t="n">
-        <v>0</v>
+        <v>1516</v>
       </c>
       <c r="I45" s="149" t="n">
-        <v>0</v>
+        <v>701</v>
       </c>
       <c r="J45" s="149" t="n">
-        <v>0</v>
+        <v>707</v>
       </c>
       <c r="K45" s="149" t="n">
-        <v>0</v>
+        <v>207</v>
       </c>
       <c r="L45" s="149" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="M45" s="149" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="N45" s="149" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="O45" s="149" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="P45" s="168" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
     </row>
     <row r="46">
@@ -18760,40 +18694,40 @@
         <v>0</v>
       </c>
       <c r="E46" s="148" t="n">
-        <v>0</v>
+        <v>1951</v>
       </c>
       <c r="F46" s="149" t="n">
-        <v>0</v>
+        <v>4890</v>
       </c>
       <c r="G46" s="149" t="n">
-        <v>0</v>
+        <v>11541</v>
       </c>
       <c r="H46" s="149" t="n">
-        <v>0</v>
+        <v>1159</v>
       </c>
       <c r="I46" s="149" t="n">
-        <v>0</v>
+        <v>606</v>
       </c>
       <c r="J46" s="149" t="n">
-        <v>0</v>
+        <v>764</v>
       </c>
       <c r="K46" s="149" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="L46" s="149" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="M46" s="149" t="n">
-        <v>0</v>
+        <v>129</v>
       </c>
       <c r="N46" s="149" t="n">
-        <v>0</v>
+        <v>113</v>
       </c>
       <c r="O46" s="149" t="n">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="P46" s="168" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
     </row>
     <row r="47">
@@ -18816,19 +18750,19 @@
         <v>0</v>
       </c>
       <c r="E47" s="148" t="n">
-        <v>0</v>
+        <v>17926</v>
       </c>
       <c r="F47" s="149" t="n">
-        <v>0</v>
+        <v>26888</v>
       </c>
       <c r="G47" s="149" t="n">
-        <v>0</v>
+        <v>51053</v>
       </c>
       <c r="H47" s="149" t="n">
-        <v>0</v>
+        <v>32321</v>
       </c>
       <c r="I47" s="149" t="n">
-        <v>0</v>
+        <v>3174</v>
       </c>
       <c r="J47" s="149" t="n">
         <v>0</v>
@@ -18864,40 +18798,40 @@
         <v>0</v>
       </c>
       <c r="E48" s="148" t="n">
-        <v>0</v>
+        <v>17926</v>
       </c>
       <c r="F48" s="149" t="n">
-        <v>0</v>
+        <v>26888</v>
       </c>
       <c r="G48" s="149" t="n">
-        <v>0</v>
+        <v>48596</v>
       </c>
       <c r="H48" s="149" t="n">
-        <v>0</v>
+        <v>92011</v>
       </c>
       <c r="I48" s="149" t="n">
-        <v>0</v>
+        <v>95765</v>
       </c>
       <c r="J48" s="149" t="n">
-        <v>0</v>
+        <v>96916</v>
       </c>
       <c r="K48" s="149" t="n">
-        <v>0</v>
+        <v>95465</v>
       </c>
       <c r="L48" s="149" t="n">
-        <v>0</v>
+        <v>86276</v>
       </c>
       <c r="M48" s="149" t="n">
-        <v>0</v>
+        <v>80878</v>
       </c>
       <c r="N48" s="149" t="n">
-        <v>0</v>
+        <v>79272</v>
       </c>
       <c r="O48" s="149" t="n">
-        <v>0</v>
+        <v>81080</v>
       </c>
       <c r="P48" s="168" t="n">
-        <v>0</v>
+        <v>82888</v>
       </c>
     </row>
     <row r="49">
@@ -18912,40 +18846,40 @@
         <v>0</v>
       </c>
       <c r="E49" s="148" t="n">
-        <v>0</v>
+        <v>17926</v>
       </c>
       <c r="F49" s="149" t="n">
-        <v>0</v>
+        <v>26888</v>
       </c>
       <c r="G49" s="149" t="n">
-        <v>0</v>
+        <v>63231</v>
       </c>
       <c r="H49" s="149" t="n">
-        <v>0</v>
+        <v>65706</v>
       </c>
       <c r="I49" s="149" t="n">
-        <v>0</v>
+        <v>67329</v>
       </c>
       <c r="J49" s="149" t="n">
-        <v>0</v>
+        <v>68510</v>
       </c>
       <c r="K49" s="149" t="n">
-        <v>0</v>
+        <v>68946</v>
       </c>
       <c r="L49" s="149" t="n">
-        <v>0</v>
+        <v>70024</v>
       </c>
       <c r="M49" s="149" t="n">
-        <v>0</v>
+        <v>70671</v>
       </c>
       <c r="N49" s="149" t="n">
-        <v>0</v>
+        <v>70024</v>
       </c>
       <c r="O49" s="149" t="n">
-        <v>0</v>
+        <v>67758</v>
       </c>
       <c r="P49" s="168" t="n">
-        <v>0</v>
+        <v>65062</v>
       </c>
     </row>
     <row r="50">
@@ -18960,40 +18894,40 @@
         <v>0</v>
       </c>
       <c r="E50" s="148" t="n">
-        <v>0</v>
+        <v>17926</v>
       </c>
       <c r="F50" s="149" t="n">
-        <v>0</v>
+        <v>26888</v>
       </c>
       <c r="G50" s="149" t="n">
-        <v>0</v>
+        <v>85605</v>
       </c>
       <c r="H50" s="149" t="n">
-        <v>0</v>
+        <v>148223</v>
       </c>
       <c r="I50" s="149" t="n">
-        <v>0</v>
+        <v>193765</v>
       </c>
       <c r="J50" s="149" t="n">
-        <v>0</v>
+        <v>181171</v>
       </c>
       <c r="K50" s="149" t="n">
-        <v>0</v>
+        <v>161710</v>
       </c>
       <c r="L50" s="149" t="n">
-        <v>0</v>
+        <v>149109</v>
       </c>
       <c r="M50" s="149" t="n">
-        <v>0</v>
+        <v>136491</v>
       </c>
       <c r="N50" s="149" t="n">
-        <v>0</v>
+        <v>128236</v>
       </c>
       <c r="O50" s="149" t="n">
-        <v>0</v>
+        <v>120245</v>
       </c>
       <c r="P50" s="168" t="n">
-        <v>0</v>
+        <v>131805</v>
       </c>
     </row>
     <row r="51">
@@ -19013,16 +18947,16 @@
         </is>
       </c>
       <c r="D51" s="116" t="n">
-        <v>0</v>
+        <v>1.037</v>
       </c>
       <c r="E51" s="148" t="n">
-        <v>0</v>
+        <v>105.5</v>
       </c>
       <c r="F51" s="266" t="n">
-        <v>0</v>
+        <v>206.6</v>
       </c>
       <c r="G51" s="267" t="n">
-        <v>0</v>
+        <v>305.2</v>
       </c>
       <c r="H51" s="148" t="n">
         <v>0</v>
@@ -19061,16 +18995,16 @@
         </is>
       </c>
       <c r="D52" s="116" t="n">
-        <v>0</v>
+        <v>1.037</v>
       </c>
       <c r="E52" s="169" t="n">
-        <v>0</v>
+        <v>105.5</v>
       </c>
       <c r="F52" s="266" t="n">
-        <v>0</v>
+        <v>206.6</v>
       </c>
       <c r="G52" s="267" t="n">
-        <v>0</v>
+        <v>305.2</v>
       </c>
       <c r="H52" s="148" t="n">
         <v>0</v>
@@ -19109,16 +19043,16 @@
         </is>
       </c>
       <c r="D53" s="116" t="n">
-        <v>0</v>
+        <v>1.037</v>
       </c>
       <c r="E53" s="267" t="n">
-        <v>0</v>
+        <v>105.5</v>
       </c>
       <c r="F53" s="266" t="n">
-        <v>0</v>
+        <v>206.6</v>
       </c>
       <c r="G53" s="267" t="n">
-        <v>0</v>
+        <v>305.2</v>
       </c>
       <c r="H53" s="148" t="n">
         <v>0</v>
@@ -19157,16 +19091,16 @@
         </is>
       </c>
       <c r="D54" s="132" t="n">
-        <v>0</v>
+        <v>1.037</v>
       </c>
       <c r="E54" s="268" t="n">
-        <v>0</v>
+        <v>105.5</v>
       </c>
       <c r="F54" s="269" t="n">
-        <v>0</v>
+        <v>206.6</v>
       </c>
       <c r="G54" s="268" t="n">
-        <v>0</v>
+        <v>305.2</v>
       </c>
       <c r="H54" s="174" t="n">
         <v>0</v>
@@ -21951,7 +21885,6 @@
     <mergeCell ref="B51:B54"/>
     <mergeCell ref="B31:B34"/>
     <mergeCell ref="B47:B50"/>
-    <mergeCell ref="A58:B58"/>
     <mergeCell ref="B27:B30"/>
     <mergeCell ref="B2:B5"/>
     <mergeCell ref="A68:A70"/>
@@ -21963,6 +21896,7 @@
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="A92:A94"/>
     <mergeCell ref="A77:A79"/>
+    <mergeCell ref="A89:A91"/>
     <mergeCell ref="A107:A109"/>
     <mergeCell ref="B19:B22"/>
     <mergeCell ref="A98:A100"/>
@@ -21988,9 +21922,9 @@
     <mergeCell ref="A95:A97"/>
     <mergeCell ref="A111:A112"/>
     <mergeCell ref="A71:A73"/>
-    <mergeCell ref="A89:A91"/>
+    <mergeCell ref="A35:A38"/>
     <mergeCell ref="A51:A54"/>
-    <mergeCell ref="A35:A38"/>
+    <mergeCell ref="A58:B58"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>